<commit_message>
added scraper project files
</commit_message>
<xml_diff>
--- a/exports/leads.xlsx
+++ b/exports/leads.xlsx
@@ -456,29 +456,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Reliance SMART Superstore</t>
+          <t>Vijay Book Depot &amp; Novelty</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>(520)</t>
+          <t>(157)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3.9(520)</t>
+          <t>4.1(157)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Hypermarket ·  · Ground &amp; 1st Floor, Plot No 1
-Open · Closes 11 pm · 1800 891 0001</t>
+          <t>Book store ·  · Shop No.17, Maurya Shopping Centre, Mulund - Airoli Link Flyover
+Open · Closes 10 pm · 080808 06575</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -486,29 +486,29 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Croma - Airoli</t>
+          <t>Morni Sarees</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(5,804)</t>
+          <t>(28)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>4.8(5,804)</t>
+          <t>3.9(28)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Electronics store ·  · Newa Bhakti Phase 1, MSEB Staff Colony, Mugalsan Rd, opposite Accenture
-Closes soon · 9 pm · Opens 11 am Mon · 086577 36964</t>
+          <t>Clothing store · Shop No -7,8,Morya Shopping Centre, -5, Navimumbai
+Open · Closes 10 pm · 091675 55399</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -516,29 +516,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Go Colors - Airoli Mumbai | Women's Bottom Wear Store</t>
+          <t>SHOPULSE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>(324)</t>
+          <t>(2)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4.8(324)</t>
+          <t>4.5(2)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Clothing store · Show Room No. 6, Ground Floor + Frist Floor, Shivshankar Plaza -1, Plot 1 Sector -8
-Closed · Opens 10 am Mon · 022 4568 9344</t>
+          <t>Clothing store · Shop No 5&amp;6
+Opens soon · 10 am · 077383 00340</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -546,169 +546,160 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Plaza Collection</t>
+          <t>Dell Exclusive Store - Mercury Towers, Airoli</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(231)</t>
+          <t>(359)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3.9(231)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>4.8(359)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Computer store · Mercury Tower, Sec B, Mulund - Airoli Rd
+Closed · Opens 11 am · 080 4800 9772</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kajri Boutique</t>
+          <t>Sagar Uniform</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>(60)</t>
+          <t>(32)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4.0(60)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>3.9(32)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Uniform store · Arihant Chs
+Open · Closes 9 pm · 098670 18921</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Westside - Bhakti Park, Airoli</t>
+          <t>Mishra General Stores</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(561)</t>
+          <t>(16)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4.0(561)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Clothing store ·  · 5XFR+284, West
-Closes soon · 9 pm · Opens 11 am Mon · 1800 209 9901</t>
-        </is>
-      </c>
+          <t>4.1(16)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Top Ten Electronics LG Shoppe, Airoli</t>
+          <t>Shopaholic</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>(228)</t>
+          <t>(52)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4.4(228)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Electronics store · Pilani CHS, Plot No C/2, Sector 3 Airoli Rd
-Open · Closes 10 pm · 093265 85747</t>
-        </is>
-      </c>
+          <t>4.0(52)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Umang Sports-Best Sports Goods &amp; Sports Wear Shop in Airoli</t>
+          <t>VARSHA WINES</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>4.3</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(47)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.3(47)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Sporting goods store · Shop No 4 Shubhrajni Society Sector 3 Opposite Airoli Railway Station, Airoli
-Open · Closes 10 pm · 086938 18779</t>
-        </is>
-      </c>
+          <t>Liquor Shop · 4XXX+9V9, Swatantryaveer Sawarkar Marg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Womaniya Airoli (Ladies western outfit shop)</t>
+          <t>Go Colors - Airoli Mumbai | Women's Bottom Wear Store</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>(232)</t>
+          <t>(324)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5.0(232)</t>
+          <t>4.8(324)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Western apparel store · Shop no 4, Eden park, plot no - 10, opposite yash paradise
-Open · Closes 10:30 pm · 090825 84301</t>
+          <t>Clothing store · Show Room No. 6, Ground Floor + Frist Floor, Shivshankar Plaza -1, Plot 1 Sector -8
+Opens soon · 10 am · 022 4568 9344</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -716,48 +707,53 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>K K Brothers (Best men’s wear in Airoli)</t>
+          <t>ASUS Exclusive Store - Icons, Airoli</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>(16)</t>
+          <t>(780)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4.9(16)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>4.8(780)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Computer store · Shop No.4, Manas Cooperative Housing Society, nearby Bank Of Baroda
+Closed · Opens 11 am · 080 3701 6397</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shopaholic</t>
+          <t>GORGEOUS WOMEN BOUTIQUE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>(52)</t>
+          <t>(27)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.0(52)</t>
+          <t>4.9(27)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -766,29 +762,29 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CottonKing Airoli</t>
+          <t>Choice Kirana Bhandar</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>(136)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4.3(136)</t>
+          <t>4.7(3)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Clothing store ·  · near Mc Donalds
-Open · Closes 10 pm · 098195 57771</t>
+          <t>Grocery store · Shop No 14, 15
+Open · Closes 10 pm · 096645 09446</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -796,31 +792,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>D Mart</t>
+          <t>Plaza Collection</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>(19,247)</t>
+          <t>(231)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4.3(19,247)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Hypermarket ·  · Dmart Rd
-Open · Closes 11 pm · 022 3340 0500</t>
-        </is>
-      </c>
+          <t>3.9(231)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -848,7 +839,7 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Clothing store ·  · Plot 2
-Open · Closes 10 pm · 098708 86392</t>
+Closed · Opens 10:30 am · 098708 86392</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -856,149 +847,129 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bittu Collection</t>
+          <t>Kajri Boutique</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>(51)</t>
+          <t>(60)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3.6(51)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Clothing store ·  · Shop No.6/7, Swami Samarth Complex, Circle, Mulund, Airoli Bridge Rd, opp. Airoli Circle, near Garam Masala Hotel
-Closes soon · 9 pm · Opens 10 am Mon · 077770 69293</t>
-        </is>
-      </c>
+          <t>4.0(60)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>The Beauty Store</t>
+          <t>Rubab The Perfect Men Shop</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>(152)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4.2(152)</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Cosmetics store ·  · Shop No. 20,21, Siddhivinayak Park CHS, near Dmart Airoli
-Open · Closes 10 pm · 088791 15599</t>
-        </is>
-      </c>
+          <t>5.0(3)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yash Electronics</t>
+          <t>Sahakar Bazar(Airoli)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>(197)</t>
+          <t>(8)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4.2(197)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Electronics wholesaler ·  · nr bank of Baroda, Yash Residency
-Open · Closes 9:30 pm · 090767 63225</t>
-        </is>
-      </c>
+          <t>3.9(8)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ninety Layers - The best Gift Shop In Airoli</t>
+          <t>SIDDHARTH KIRANA &amp;GENERAL STORE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(39)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4.9(39)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Gift shop · Shop no 3, Gaothan Sector 20 Airoli Rd
-Open · Closes 10 pm · 086918 12883</t>
-        </is>
-      </c>
+          <t>4.2(5)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ASUS Exclusive Store - Icons, Airoli</t>
+          <t>Parison</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>(780)</t>
+          <t>(13)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4.8(780)</t>
+          <t>4.2(13)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Computer store · Shop No.4, Manas Cooperative Housing Society, nearby Bank Of Baroda
-Closes soon · 8:30 pm · Opens 11 am Mon · 080 3701 6397</t>
+          <t>Clothing store · Vraj Vihar CHS, Mugalsan Rd
+Open · Closes 10:30 pm · 090293 43643</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1006,31 +977,26 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cotton Culture</t>
+          <t>Jay par maa super market</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(249)</t>
+          <t>(38)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4.9(249)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Clothing store · Shop No. 11, Chs Ltd, Cotton Culture, Plot No. 53
-Open · Closes 10 pm · 093727 09143</t>
-        </is>
-      </c>
+          <t>3.4(38)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1058,7 +1024,7 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>Clothing store · Shop No.13, Airoli Plaza A, Plot No.04
-Open · Closes 10 pm · 098671 55595</t>
+Opens soon · 10 am · 098671 55595</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1066,29 +1032,29 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jockey Exclusive Store</t>
+          <t>Womaniya Airoli (Ladies western outfit shop)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(3,039)</t>
+          <t>(232)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4.8(3,039)</t>
+          <t>5.0(232)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Clothing store ·  · Shop No 9, Plot No 1, 1A, 1B, Shivshankar Plaza 1, near Mc Donald
-Open · Closes 9:30 pm · 085919 04552</t>
+          <t>Western apparel store · Shop no 4, Eden park, plot no - 10, opposite yash paradise
+Closed · Opens 12 pm · 090825 84301</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1096,29 +1062,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Parison</t>
+          <t>St Raphael Store</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>(13)</t>
+          <t>(11)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>4.2(13)</t>
+          <t>3.2(11)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Clothing store · Vraj Vihar CHS, Mugalsan Rd
-Open · Closes 10 pm · 090293 43643</t>
+          <t>General store · Shop Number 57, Yash Pradise, Sector Number 8a
+Open · Closes 10 pm · 098219 86470</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1126,29 +1092,29 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Airoli brands factory</t>
+          <t>Ambaji Enterprises</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(3)</t>
+          <t>(11)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>5.0(3)</t>
+          <t>4.4(11)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Clothing store · K-2, 400708, near Kasturi garden building
-Open · Closes 11 pm · 089282 53353</t>
+          <t>Stationery store · plot no-1889, Shop no-1/2 Opp to Rakesh kabra and Co. T.T.C. Industrial Area, bhimnagar
+Open · Closes 9 pm · 098704 51111</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1156,29 +1122,29 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Vastra Ghar Family Shop</t>
+          <t>Hari Om Dairy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>(13)</t>
+          <t>(103)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4.4(13)</t>
+          <t>4.0(103)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Clothing store · Shop No.1,2
-Open · Closes 10 pm · 098197 21722</t>
+          <t>Dairy store · SS2-N/16
+Open · Closes 11 pm · 099207 12718</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1186,29 +1152,29 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>POORNIMA ELECTRIC &amp; &amp; HARDWARE STORES</t>
+          <t>Purnima Super Market</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(485)</t>
+          <t>(8)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>4.1(485)</t>
+          <t>3.6(8)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Hardware store ·  · Shop No.5,6,7
-Open · Closes 10 pm · 077389 35555</t>
+          <t>General store · Shop Number 5 Plot Number 64, Sector 8A
+Open · Closes 11 pm · 092210 67729</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1216,23 +1182,23 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Peshwai A fashion destination &amp; Ethnic Shop</t>
+          <t>Aastha Communication</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>(13)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4.7(13)</t>
+          <t>5.0(1)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1241,29 +1207,29 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lenovo Exclusive Store - Absolute It Solutions</t>
+          <t>Bittu Collection</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(620)</t>
+          <t>(51)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>4.9(620)</t>
+          <t>3.6(51)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Computer store · Plot No.4, Shop No.2 Mercury Co-op Housing Society
-Closes soon · 9 pm · Opens 11 am Mon · 080 4807 2448</t>
+          <t>Clothing store ·  · Shop No.6/7, Swami Samarth Complex, Circle, Mulund, Airoli Bridge Rd, opp. Airoli Circle, near Garam Masala Hotel
+Opens soon · 10 am · 077770 69293</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1271,29 +1237,29 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Shreeji Super Market</t>
+          <t>RADHA SWAMI GENERAL STORES</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>(441)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>4.3(441)</t>
+          <t>5.0(1)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Grocery store · 
-Closes soon · 9 pm · Opens 9:30 am Mon · 088501 08001</t>
+          <t>Store · PLOT R, PAP, 69, Rabale MIDC Rd, near SAI PRASAD HOTEL
+Open · Closes 11:30 pm · 097685 27286</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1301,23 +1267,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mishra General Stores</t>
+          <t>Peshwai A fashion destination &amp; Ethnic Shop</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(16)</t>
+          <t>(13)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>4.1(16)</t>
+          <t>4.7(13)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1326,29 +1292,29 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Vighnahar Electronics</t>
+          <t>Navi Mumbai Matching Center</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>(40)</t>
+          <t>(10)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4.5(40)</t>
+          <t>4.2(10)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Electronics store · Shop no. 7, Divagaon
-Open · Closes 9:30 pm · 081085 38589</t>
+          <t>Fabric store · Shop No 24, shree Ganesh market, near Radikabai meghe school
+Opens soon · 10 am · 090047 04490</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1381,29 +1347,29 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Classy Style | Mens | Women's Wear Shop In Airoli | Multi Brands Clothes In Airoli</t>
+          <t>Sai Sweet Mart</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(5)</t>
+          <t>(10)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>4.2(5)</t>
+          <t>3.6(10)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Clothing store · Shop No. 8, Shivshankar Plaza 1, Chs. Ltd
-Open · Closes 9:30 pm · 093218 92226</t>
+          <t>Sweet shop · Shop no-430, Near Ekta Vidyalay, Thane-Belapur Road, Bhim Nagar, Rabale
+Open · Closes 10:30 pm · 099208 42763</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -1411,29 +1377,29 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mauli Sports</t>
+          <t>Suvidha General Stores</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(228)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4.2(228)</t>
+          <t>3.7(3)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sporting goods store ·  · Shop no 8 plot no, Sagar CHS, Shree Sai Apartment, B-8/9, near Garam Masala Hotel
-Open · Closes 9:30 pm · 088793 27676</t>
+          <t>General store · Shop No. 6, 5X2V+VQ5
+Open · Closes 10:30 pm · 093246 90090</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -1441,29 +1407,29 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>The Helmet Store</t>
+          <t>Bhonaji Super Market</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>(179)</t>
+          <t>(15)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>4.1(179)</t>
+          <t>4.8(15)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Helmet Shop ·  · Shop No.1, Near, Mulund - Airoli Rd
-Closes soon · 9 pm · Opens 11 am Mon · 091677 65751</t>
+          <t>Grocery store · 4XRW+GRR
+Open · Closes 11 pm · 087677 99555</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -1471,29 +1437,29 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vijay Book Depot &amp; Novelty</t>
+          <t>Titan Eye+ at Airoli, Navi Mumbai (Buy 1 Get 1 Free)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(157)</t>
+          <t>(188)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>4.1(157)</t>
+          <t>4.8(188)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Book store ·  · Shop No.17, Maurya Shopping Centre, Mulund - Airoli Link Flyover
-Open · Closes 10 pm · 080808 06575</t>
+          <t>Optician · Floor, and First Floor, Shivshankar Plaza, Shop No. G-14, on Ground, Plot No 1
+Closed · Opens 10:30 am · 082912 66296</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -1501,23 +1467,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Airoli Sector 4 Siddhakala Stores</t>
+          <t>Nadar Kirana Store</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>(39)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>3.8(39)</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -1526,29 +1492,29 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Profit Point</t>
+          <t>PURPLE ROSE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(6)</t>
+          <t>(9)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>3.7(6)</t>
+          <t>3.4(9)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Clothing store · Shop Number 4 Plot Number 4, Sector 3 Airoli Rd
-Open · Closes 10 pm · 070574 67656</t>
+          <t>Clothing store · Shop no-8-9, opposite Mcdonald's
+Opens soon · 10 am · 082867 28333</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -1556,29 +1522,29 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Shree Ram Mobile - Mobile Phone dealer in Airoli</t>
+          <t>MILAP GENERAL STORE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>(221)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>4.7(221)</t>
+          <t>3.4(5)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Cell phone store ·  · Shop No 17
-Open · Closes 10:30 pm · 077100 26886</t>
+          <t>General store · Shop No 01
+097630 65911</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -1586,30 +1552,29 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bake Ur Day a Custom Cakery - Cake Shop in Airoli</t>
+          <t>A1 CHICKEN CENTER</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(888)</t>
+          <t>(98)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4.4(888) · ₹200–1,200</t>
+          <t>3.9(98)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Cake shop ·  · Shop No. 3, Airoli Tower Rd, opp. Gaodevi Maidan, Airoli
-Bakery preparing occasion cakes
-Open · Closes 1 am · 090048 88063</t>
+          <t>Bakery and Cake Shop · AL-1/246
+Open · Closes 11 pm · 083696 48731</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -1617,59 +1582,54 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LA Home decor &amp; gifts</t>
+          <t>Laxmi narayan Dairy n icecreams</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>(13)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4.5(13)</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Gift shop · shop no 3, Goodwill Harmony, 16
-Open · Closes 10:30 pm · 080800 53678</t>
-        </is>
-      </c>
+          <t>3.7(3)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Poojara Telecom, Airoli (Best Mobile Phone Experience store in Navi Mumbai)</t>
+          <t>Sanskruti Silk &amp; Designer Sarees</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(63)</t>
+          <t>(22)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>4.9(63)</t>
+          <t>4.0(22)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Cell phone store · shop 6, Airoli Plaza B
-Open · Closes 10 pm · 088792 28447</t>
+          <t>Clothing store · 6, Om Shivdarshan CHS, Acharya Vinobha Bhave Rd, opp. Saraswat Bank
+Open · Closes 10 pm · 022 2769 6785</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -1677,7 +1637,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Karishma Beer Shop</t>
+          <t>New Gift Galleria</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -1688,18 +1648,18 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(257)</t>
+          <t>(9)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>4.0(257)</t>
+          <t>4.0(9)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Beer store ·  · Saptagiri Apartment, Plot No.1, Shop No.7, Diva Nagar Rd
-Open · Closes 11 pm · 096194 46565</t>
+          <t>Gift shop · Shop Numbar 3 Plot Number 2 Shashwat Co- Op Sector 8 A
+Open · Closes 10 pm · 099200 67118</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -1707,38 +1667,43 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>New gifteria</t>
+          <t>Vitthal Pan Centre</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(32)</t>
+          <t>(247)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>3.2(32)</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
+          <t>4.5(247) · ₹1–200</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Paan shop ·  · 4XXR+G75
+Open · Closes 11 pm · 098331 82521</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PURPLE ROSE</t>
+          <t>RAMESHWAR KIRANA STORES</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>4.9</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1748,13 +1713,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>3.4(9)</t>
+          <t>4.9(9)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Clothing store · Shop no-8-9, opposite Mcdonald's
-Open · Closes 10 pm · 082867 28333</t>
+          <t>Grocery store · Rameshwar kirana stors, gali, near Narayan furniture
+Open · Closes 11 pm · 090042 25004</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -1762,29 +1727,29 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Stationery Point Gift and Toy</t>
+          <t>Maharashtra Shopping</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(34)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>4.8(34)</t>
+          <t>3.0(1)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Toy store · Shop no 44, yash Paradise
-Open · Closes 10:30 pm · 086522 31439</t>
+          <t>Store ·  · Gate Number D
+Open · Closes 6 am Tue · 070392 44746</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -1792,29 +1757,29 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Thakkar Fones</t>
+          <t>Style Men's Wear</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>(94)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4.3(94)</t>
+          <t>3.8(5)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Cell phone store · near kesar sweets
-Open · Closes 10 pm · 080972 09728</t>
+          <t>Clothing store · J-190, Airoli Station Main Rd, opp. Mahanagar Palika Office
+Open · Closes 9:30 pm · 097025 55715</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -1822,29 +1787,29 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Lenskart</t>
+          <t>B Mart</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>(979)</t>
+          <t>(176)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>4.5(979)</t>
+          <t>4.4(176)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Optician ·  · Shop No G9, Shivshankar Plaza 2, G9, Mulund - Airoli Rd, next to Dominos Pizza
-Open · Closes 10 pm · 074288 91243</t>
+          <t>Grocery store · Plot No. 7, Sector 11, Shop No.27,28,29 Gold Crest Recidency, New, Palm Beach Rd, near Cloud 36
+Open · Closes 9:30 pm · 079772 77468</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -1852,29 +1817,29 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Navi Mumbai Matching Center</t>
+          <t>Suraj Grocery Shop</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(10)</t>
+          <t>(11)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>4.2(10)</t>
+          <t>4.8(11)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Fabric store · Shop No 24, shree Ganesh market, near Radikabai meghe school
-Open · Closes 10 pm · 090047 04490</t>
+          <t>Supermarket · Datt Nagar Ghansoli , Near mari aai chowk, R/N:-001/124
+Open · Closes 10 pm · 086554 50678</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -1882,84 +1847,84 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PATIL WINES</t>
+          <t>Popular Furnishing</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>(318)</t>
+          <t>(37)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>4.5(318)</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>4.6(37)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Curtain supplier and maker ·  · shop.no.6, co op society, 6a
+Closed · Opens 10 am Tue · 098207 96276</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>New Gift Galleria</t>
+          <t>A To Z Boutique</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>(9)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>4.0(9)</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Gift shop · Shop Numbar 3 Plot Number 2 Shashwat Co- Op Sector 8 A
-Open · Closes 10 pm · 099200 67118</t>
-        </is>
-      </c>
+          <t>5.0(1)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Theobroma Bakery and Cake Shop - Airoli, Navi Mumbai</t>
+          <t>Kanhaiya Kids Wear</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>(110)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>3.4(110) · ₹200–1,000</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Cake shop · Shop No 3 &amp; 4, Ground Floor, Ramdas Apartment
-Open · Closes 11 pm · 081828 81881</t>
+          <t>Clothing store · Shop Number 18, Plot, 18, Sector 3 Airoli Rd
+Open · Closes 10:30 pm · 097686 23047</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -1967,29 +1932,29 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>New poornima electric &amp; hardware stores</t>
+          <t>Mujeeb Mutton And Chicken Shop</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>(40)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>4.2(40)</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Building materials store · Shop No.4B
-Open · Closes 10 pm · 082600 03939</t>
+          <t>Chicken &amp; Mutton Shop · 42V3+RCC, Thane - Belapur Rd
+Open · Closes 7:30 pm · 090042 78886</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -1997,59 +1962,54 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Chetak Sweet Point Airoli</t>
+          <t>A To Z General Store</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>(920)</t>
+          <t>(61)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4.7(920) · ₹₹</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Indian sweets shop · Shop no 12, Vraj Vihar Complex, CHS ltd, Plot no 5
-Open · Closes 10:30 pm · 090043 33322</t>
-        </is>
-      </c>
+          <t>4.2(61)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Star Electrovision</t>
+          <t>Maharashtra Society Stores</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>(276)</t>
+          <t>(42)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>4.9(276)</t>
+          <t>4.3(42)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Electronics store · Shop No. 3, Marathon Corner, Sector 3 Airoli Rd
-Open · Closes 9:30 pm · 092247 43638</t>
+          <t>Grocery store ·  · Shop No. 4, Shreenath Apt, 2, Chafekar Bandhu Marg
+Open · Closes 10 pm · 093242 41298</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -2057,29 +2017,29 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KisanKonnect Farm Store-Airoli</t>
+          <t>ELITE LADIES FASHION</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>(59)</t>
+          <t>(2)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>3.9(59)</t>
+          <t>3.0(2)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Produce market · Plot No.09, Shop No 14, Opposite: Yash Paradise
-Open · Closes 11 pm · 1800 267 0997</t>
+          <t>Women's clothing store · Shop No 9, Plot No 21, Krishna Kanhaiya Co.Op.Hsg Society Ltd
+Closed · Opens 11 am · 096648 06520</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -2087,54 +2047,56 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Airoli chinchpada Ganesh Nagar</t>
+          <t>Diamond Kirana Store</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>(20)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>4.7(20)</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>5.0(5)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>General store · Shop H 22, Rupa Kumar Vaidya Marg, Sector 3 Airoli Rd
+Open · Closes 11 pm · 099205 75749</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NEW SWASTIK STORES</t>
+          <t>Mahak Collection</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>(4)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>5.0(4)</t>
+          <t>Clothing store · Shop No. 1, Janaki CHS
+081088 09690</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>General store · AL/1/495, Sector 16
-Open · Closes 10:30 pm · 093222 88881</t>
+          <t>Clothing store · Shop No. 1, Janaki CHS
+081088 09690</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -2142,29 +2104,29 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Kumar Collection Men’s airoli - All varieties of Best Kurta, Blazer Suits , Jodhpuri , Sherwani ,Formals</t>
+          <t>ASHAPURA KIRANA AND GENERAL STORE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>(27)</t>
+          <t>(11)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4.5(27)</t>
+          <t>3.7(11)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Men's clothing store · Shop No.3, Mehul Apartment, Arun Kumar Vidhya Marg, next to shakuntala hospital
-Open · Closes 10 pm · 090291 02004</t>
+          <t>Supermarket · R-1, Dead Rd
+Open · Closes 10:30 pm · 098194 31772</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
@@ -2172,29 +2134,29 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Vitthal Pan Centre</t>
+          <t>VARSHA FURNISHING</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>(247)</t>
+          <t>(16)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>4.5(247) · ₹1–200</t>
+          <t>4.6(16)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Paan shop ·  · 4XXR+G75
-Open · Closes 11 pm · 098331 82521</t>
+          <t>Furniture store · Shop No. 13, Shree Gurudatta Complex, Chs Ltd
+098929 54338</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -2202,23 +2164,23 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Sugee General Stores</t>
+          <t>Rohit Kirana Store</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>(27)</t>
+          <t>(12)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>4.6(27)</t>
+          <t>4.2(12)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2227,29 +2189,29 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Maitreen Mobile</t>
+          <t>A-One General Store</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>(32)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>4.3(32)</t>
+          <t>5.0(1)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Cell phone store · Space Plaza, Shop No -6, 'B',Sector -16,Airoli,Navimumbai
-Open · Closes 10 pm · 080802 02076</t>
+          <t>Grocery store · Plot No. 614, Shivam society, Shop No. 6
+Open · Closes 11 pm · 097028 84608</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -2257,29 +2219,29 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SHOPULSE</t>
+          <t>Style Men's Wear</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>(2)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>4.5(2)</t>
+          <t>3.8(5)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Clothing store · Shop No 5&amp;6
-Closes soon · 9 pm · Opens 10 am Mon · 077383 00340</t>
+          <t>Clothing store · J-190, Airoli Station Main Rd, opp. Mahanagar Palika Office
+Open · Closes 9:30 pm · 097025 55715</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
@@ -2287,29 +2249,29 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Prabhat Sports</t>
+          <t>Popular Furnishing</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>(9)</t>
+          <t>(37)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4.8(9)</t>
+          <t>4.6(37)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Sportswear store · Shop No, B78, Sector 3 Airoli Rd
-Open · Closes 11 pm · 080802 18200</t>
+          <t>Curtain supplier and maker ·  · shop.no.6, co op society, 6a
+Closed · Opens 10 am Tue · 098207 96276</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
@@ -2317,29 +2279,29 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Chamunda Stationery And Novelty Stores</t>
+          <t>Kanhaiya Kids Wear</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>(58)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4.4(58)</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Stationery store ·  · Shop No: 1, Plot No: 26, Ganesh Market
-Open · Closes 10 pm · 091677 18818</t>
+          <t>Clothing store · Shop Number 18, Plot, 18, Sector 3 Airoli Rd
+Open · Closes 10:30 pm · 097686 23047</t>
         </is>
       </c>
       <c r="G66" t="inlineStr"/>
@@ -2347,89 +2309,79 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>90 Degrees - The Cake Studio</t>
+          <t>A To Z Boutique</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>(524)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>4.9(524) · ₹200–1,000</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Cake shop · Shop No. 06, Marathon Vastu
-Open · Closes 12 am · 088798 09090</t>
-        </is>
-      </c>
+          <t>5.0(1)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Gami general store</t>
+          <t>A To Z General Store</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>(10)</t>
+          <t>(61)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>4.4(10)</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>General store · Shop no A33, Sector 3 Airoli Rd
-Open · Closes 10 pm · 090767 67624</t>
-        </is>
-      </c>
+          <t>4.2(61)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>HP World - Airoli</t>
+          <t>Maharashtra Society Stores</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>(52)</t>
+          <t>(42)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>4.5(52)</t>
+          <t>4.3(42)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Computer store · Shop No 3, Ground Floor, Manas Cooperative Housing Society, Plot No 5
-Closes soon · 9 pm · Opens 11 am Mon · 088799 74941</t>
+          <t>Grocery store ·  · Shop No. 4, Shreenath Apt, 2, Chafekar Bandhu Marg
+Open · Closes 10 pm · 093242 41298</t>
         </is>
       </c>
       <c r="G69" t="inlineStr"/>
@@ -2437,7 +2389,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Airoli Furnishing And Handloom</t>
+          <t>Mujeeb Mutton And Chicken Shop</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
@@ -2448,18 +2400,18 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>(2)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>5.0(2)</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Clothing store · Shop No. 5, Sant Sawata Bhawan, Plot No. 31, Sector 5, Airoli, Station Road, Airoli Navi Mumbai
-Open · Closes 10 pm · 098191 45757</t>
+          <t>Chicken &amp; Mutton Shop · 42V3+RCC, Thane - Belapur Rd
+Open · Closes 7:30 pm · 090042 78886</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
@@ -2467,29 +2419,29 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>geeta emporium</t>
+          <t>Shree Ganesh Kirana Ghar</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>(2)</t>
+          <t>(7)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>4.0(2)</t>
+          <t>4.3(7)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Clothing store · shop no.A-6, super market
-Open · Closes 9:30 pm · 091679 00925</t>
+          <t>General store · 5X2R+5QJ
+Open · Closes 10:30 pm · 098709 15223</t>
         </is>
       </c>
       <c r="G71" t="inlineStr"/>
@@ -2497,29 +2449,29 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Shree Hari Krishna-Furniture Shop in Airoli</t>
+          <t>Bhilare Brothers Men's Corner</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>(37)</t>
+          <t>(8)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>3.5(37)</t>
+          <t>4.5(8)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Furniture store · Branch &amp; ATM, Shop No -03.4 &amp; 5,Riddling Siddhi Hreitage Plot No-57,Section 19, near ICICI Bank
-Open · Closes 9:30 pm · 022 2779 4477</t>
+          <t>Sportswear store · Gala No. 1, Bhilare Brothers Men's Corner, near Chintamani Hotel Elthanpada
+Open · Closes 10:30 pm · 083697 06128</t>
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
@@ -2527,29 +2479,29 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Shree Yash Bag Center</t>
+          <t>Diamond Kirana Store</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>(31)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>4.6(31)</t>
+          <t>5.0(5)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Bag shop · H, shop, 258, Rajrishi Shahu Maharajah Marg
-Open · Closes 9:30 pm · 090042 93300</t>
+          <t>General store · Shop H 22, Rupa Kumar Vaidya Marg, Sector 3 Airoli Rd
+Open · Closes 11 pm · 099205 75749</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
@@ -2557,29 +2509,29 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SSD Mobile Gallery</t>
+          <t>ELITE LADIES FASHION</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>(147)</t>
+          <t>(2)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>4.5(147)</t>
+          <t>3.0(2)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Cell phone store · Shop No 22, Madhuri Tower, near KFC
-Open · Closes 11 pm · 098679 33655</t>
+          <t>Women's clothing store · Shop No 9, Plot No 21, Krishna Kanhaiya Co.Op.Hsg Society Ltd
+Closed · Opens 11 am · 096648 06520</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
@@ -2587,29 +2539,26 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Titan Eye+ at Airoli, Navi Mumbai (Buy 1 Get 1 Free)</t>
+          <t>Mahak Collection</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>4.8</t>
-        </is>
-      </c>
+      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>(188)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>4.8(188)</t>
+          <t>Clothing store · Shop No. 1, Janaki CHS
+081088 09690</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Optician · Floor, and First Floor, Shivshankar Plaza, Shop No. G-14, on Ground, Plot No 1
-Open · Closes 9:30 pm · 082912 66296</t>
+          <t>Clothing store · Shop No. 1, Janaki CHS
+081088 09690</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
@@ -2617,29 +2566,29 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Glorious Sports Airoli</t>
+          <t>Jai Gurudev Kirana Store</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>(7)</t>
+          <t>(20)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>5.0(7)</t>
+          <t>3.6(20)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Clothing store
-096643 39312</t>
+          <t>General store · 400708
+Open · Closes 10 pm · 096997 87906</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
@@ -2647,29 +2596,29 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Step In Shoes</t>
+          <t>VARSHA FURNISHING</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>(24)</t>
+          <t>(16)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>3.6(24)</t>
+          <t>4.6(16)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Shoe store · Shop no.8, shreeji dham, plot no 7
-Open · Closes 10 pm · 095949 36089</t>
+          <t>Furniture store · Shop No. 13, Shree Gurudatta Complex, Chs Ltd
+098929 54338</t>
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
@@ -2677,7 +2626,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MedPlus Airoli Sector 8</t>
+          <t>Low Price</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
@@ -2688,48 +2637,40 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>(5)</t>
+          <t>(304)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>4.2(5)</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Pharmacy · Shop C22, Shree Gurudatta Complex, Acharya V Bhave Road
-Open · Closes 11 pm · 040 6700 6700</t>
-        </is>
-      </c>
+          <t>4.2(304)</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SM MARBLES</t>
+          <t>Shreyash Medical &amp; General Stores</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>4.3</t>
-        </is>
-      </c>
+      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>(4)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>4.3(4)</t>
+          <t>Medical Center · Shop Number 92, Jai Jawan Apartment, AL-1/96
+Opens soon · 10 am · 072080 44616</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Men's clothing store · Shop No.15, Super Market, Bharatratna Ambedkar Rd
-Closed · Opens 9 am Mon · 098700 98531</t>
+          <t>Medical Center · Shop Number 92, Jai Jawan Apartment, AL-1/96
+Opens soon · 10 am · 072080 44616</t>
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
@@ -2737,29 +2678,29 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Clothing King</t>
+          <t>ASHAPURA KIRANA AND GENERAL STORE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>(5)</t>
+          <t>(11)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>4.2(5)</t>
+          <t>3.7(11)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Clothing store · behind SDV College
-Closed · Opens 10:30 am Mon · 091368 01443</t>
+          <t>Supermarket · R-1, Dead Rd
+Open · Closes 10:30 pm · 098194 31772</t>
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
@@ -2767,29 +2708,29 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Kailash Kirana Shop</t>
+          <t>Rajesh super market</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>(11)</t>
+          <t>(2)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>4.5(11)</t>
+          <t>5.0(2)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Supermarket · SS3-A/23, Koparkar Marg
-Open · Closes 10 pm · 099878 57806</t>
+          <t>Supermarket · Shop no 11 Sec 2 Plot no 127 Ulwe Node
+Open · Closes 11 am · 084540 92736</t>
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
@@ -2797,67 +2738,53 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Techno Shop</t>
+          <t>Ramesh kirana stores</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>(132)</t>
+          <t>(2)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>3.9(132)</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Cell phone store ·  · Mulund - Airoli Link Flyover
-Open · Closes 10 pm · 097733 64444</t>
-        </is>
-      </c>
+          <t>5.0(2)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Bata Shop</t>
+          <t>VARSHA WINES</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>3.7</t>
-        </is>
-      </c>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>(108)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3.7(108)</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Clothing store · Mulund - Airoli Link Flyover
-Closes soon · 9 pm · Opens 11 am Mon · 099705 57355</t>
-        </is>
-      </c>
+          <t>Liquor Shop · 4XXX+9V9, Swatantryaveer Sawarkar Marg</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Cambridge readymades</t>
+          <t>Mujeeb Mutton And Chicken Shop</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -2868,43 +2795,48 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>(4)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>5.0(4)</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
+          <t>5.0(3)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Chicken &amp; Mutton Shop · 42V3+RCC, Thane - Belapur Rd
+Open · Closes 7:30 pm · 090042 78886</t>
+        </is>
+      </c>
       <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Shoe Museum</t>
+          <t>Variya Super Shop</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>(16)</t>
+          <t>(6)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>3.3(16)</t>
+          <t>4.0(6)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Shoe store · Shop No -12, Airoli Plaza B
-Open · Closes 10 pm · 091675 76575</t>
+          <t>Grocery store · Shop No-2, Gavanpada Rd
+Open · Closes 10 pm · 098678 69733</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
@@ -2912,29 +2844,29 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Sai Book Depot &amp; General Store</t>
+          <t>Milan General Stores</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>(442)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>4.2(442)</t>
+          <t>5.0(5)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Book store ·  · Rh.4, Sundervan Co. Operative Housing Society., opp. Datta Meghe Engn College
-Closes soon · 9 pm · Opens 10 am Mon · 097697 60097</t>
+          <t>General store · Shop no- 8 , Vity Bhavan,, Chaphekar Road, Nav Indraprastha CHS, Mulund East
+Closed · Opens 8:30 am Tue · 083697 91254</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -2942,7 +2874,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Kekiz - The Cake Shop Airoli</t>
+          <t>Big toy world 🌎 Mumbra wholesaler &amp; retailer</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -2953,18 +2885,18 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>(47)</t>
+          <t>(92)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>4.9(47)</t>
+          <t>4.9(92)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Cake shop · Shop No.2, Regina CHS, Plot No. 18
-Open · Closes 11 pm · 084240 93288</t>
+          <t>Toy store · near Abdullah Patel English school
+Closed · Opens 11 am · 096196 83313</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
@@ -2972,114 +2904,106 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Apollo Pharmacy Airoli Sector 8</t>
+          <t>Vaity Shop</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>(52)</t>
+          <t>(3)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>4.4(52)</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Pharmacy · Ground Floor, Dattatraya Maharaj Society, Plot No.6, Shop No.3&amp;4
-Open 24 hours · 079 4747 9503</t>
-        </is>
-      </c>
+          <t>4.7(3)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sagar Uniform</t>
+          <t>R Retailers</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>(32)</t>
+          <t>(5)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>3.9(32)</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Uniform store · Arihant Chs
-Closes soon · 9 pm · Opens 9 am Mon · 098670 18921</t>
-        </is>
-      </c>
+          <t>5.0(5)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Mahalaxmi Jewellers</t>
+          <t>Society Super Market</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>(176)</t>
+          <t>(7)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>4.0(176)</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr"/>
+          <t>4.6(7)</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>General store · Rambhau Mhalgi Rd
+Closed · Opens 8 am Tue · 081691 02028</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CELL CITY</t>
+          <t>Maharashtra General Stores</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>3.9</t>
-        </is>
-      </c>
+      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
-          <t>(134)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>3.9(134)</t>
+          <t>General store · 5XFX+9FX, Thane - Belapur Rd
+Open · Closes 10:30 pm · 084332 59216</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Cell phone store · Shop no 9, Rajkamal Chs, Sector 3 Airoli Rd
-Open · Closes 10:30 pm · 077382 21213</t>
+          <t>General store · 5XFX+9FX, Thane - Belapur Rd
+Open · Closes 10:30 pm · 084332 59216</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -3087,29 +3011,29 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Zeelab Pharmacy - Airoli</t>
+          <t>Daily Mart</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>(474)</t>
+          <t>(12)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>4.9(474)</t>
+          <t>4.4(12)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Pharmacy · SHOP NO. H-163, GROUND FLOOR, Sector 3 Airoli Rd
-Open · Closes 11 pm · 098962 77748</t>
+          <t>Grocery store · 5WFX+3X4 Kailash Ashish Tower, 07, Dr Ambedkar Rd, opp. Kalidas Cmplx
+Open · Closes 9:30 pm · 079778 25454</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
@@ -3117,29 +3041,26 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Jai Gurudev Kirana Store</t>
+          <t>Devika Supermarket</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>3.6</t>
-        </is>
-      </c>
+      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>(20)</t>
+          <t>No reviews</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>3.6(20)</t>
+          <t>General store · Shop No 1, Hari Om Nagar Rd
+Open · Closes 10 pm · 081695 67332</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>General store · 400708
-Open · Closes 10 pm · 096997 87906</t>
+          <t>General store · Shop No 1, Hari Om Nagar Rd
+Open · Closes 10 pm · 081695 67332</t>
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
@@ -3147,59 +3068,54 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>The Ice Cream Bakery, Airoli</t>
+          <t>Aastha Communication</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>(836)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>4.3(836) · ₹₹</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Ice Cream ·  · Shop No G8 &amp; G9, Ripplez Mall, Plot No.6A, near McDonald's
-Open · Closes 1 am · 088983 63087</t>
-        </is>
-      </c>
+          <t>5.0(1)</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ALL IN ONE SUPPLIERS PVT. LTD.</t>
+          <t>ASHAPURA PROVISION STORE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>(21)</t>
+          <t>(1)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>4.6(21)</t>
+          <t>2.0(1)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Plywood supplier ·  · Plot No.19, Sector 4, Thane Belapur Road, Airoli
-Closed · Opens 10 am Mon · 070459 43848</t>
+          <t>Bicycle Shop · Shop No 1, Airoli Gaon Gali
+095617 44622</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>

</xml_diff>